<commit_message>
atlanta-basement-design: workbook guardrail notes rewritten in client voice
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/atlanta-basement-design/keyword-research.xlsx
+++ b/decks/atlanta-basement-design/keyword-research.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>SERVICE PAGE REBUILD - /custom-basement-bars is 206 words today. Cost language must follow brand-facts.md: specialty finishes sit on top of the $45k-$80k basic construction range.</t>
+          <t>Rebuild of your existing bars page, which runs 206 words today. Any cost figures use your own published ranges, with specialty finishes shown as sitting on top of the $45,000 to $80,000 basic construction range.</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>SERVICE PAGE REBUILD - /home-theaters is 195 words today.</t>
+          <t>Rebuild of your existing home theaters page, which runs 195 words today.</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>SERVICE PAGE REBUILD - /ceilings is 188 words today.</t>
+          <t>Rebuild of your existing ceilings page, which runs 188 words today.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>SERVICE PAGE REBUILD - /exterior-remodeling is 210 words today.</t>
+          <t>Rebuild of your existing exterior remodeling page, which runs 210 words today.</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Coverage play. Must carry Gwinnett County permit detail and real local projects, not a template spin.</t>
+          <t>No measured search volume, so this is coverage rather than a traffic play. Carries Gwinnett County permit detail and real projects in the area, not a reworded template.</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Cobb County permit detail required.</t>
+          <t>No measured search volume. Carries Cobb County permit detail.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Newton County. Check 30-mile warranty radius from Marietta.</t>
+          <t>No measured search volume. Newton County. We will confirm Covington sits inside your 30-mile service radius before writing it.</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Clayton County.</t>
+          <t>No measured search volume. Clayton County.</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Clayton County.</t>
+          <t>No measured search volume. Clayton County.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Zero measured volume. Fulton County.</t>
+          <t>No measured search volume. Fulton County.</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>HOLD until Judith confirms Griffin is inside the 30-mile warranty radius. Spalding County.</t>
+          <t>On hold until you confirm Griffin falls inside the 30-mile radius your warranty covers. Spalding County.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>HOLD until Judith confirms Hampton is inside the 30-mile warranty radius. Henry County.</t>
+          <t>On hold until you confirm Hampton falls inside the 30-mile radius your warranty covers. Henry County.</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Must reflect brand-facts.md hedging: 'routinely the lowest bid', never 'guaranteed lowest'.</t>
+          <t>Uses your own wording, "routinely the lowest bid our clients receive". Never hardened into a guarantee.</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Differentiation angle. Green Basements is a generalist who added basements - this is the honest wedge.</t>
+          <t>A differentiation piece. Makes the case for a basement specialist on the merits, without naming or disparaging any competitor.</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Anchors the 'Real Pricing, No Surprises' positioning. Structural-change exception must appear.</t>
+          <t>Extends your Real Pricing, No Surprises page. States plainly that major structural changes are the exception to your no-upcharge position.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Do NOT publish a license number - none is published on the live site.</t>
+          <t>Describes your team as licensed with 20-plus years per trade, matching your About page. No license number appears, because your site does not publish one and we only state what you have stated.</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>3D CAD design and the on-site pre-quote visit are verified in brand-facts.md.</t>
+          <t>Built on two things your site already states: the custom 3D CAD design, and the on-site visit before any quote.</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>FLAGGED: must present $45-$150/sq ft as a range and separate basic construction from specialty finishes.</t>
+          <t>Presents your published $45 to $150 per square foot as a range, and keeps basic construction separate from specialty finishes.</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Generic financing education only. ABD does not offer financing - do not imply an in-house program.</t>
+          <t>General guidance on how homeowners fund a basement, written so it never implies you offer financing yourself.</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>FLAGGED: ABD's own 70-80% ROI figure needs a third-party source alongside it.</t>
+          <t>Your FAQ puts the Atlanta return at 70 to 80 percent. This article carries an independent source alongside that figure rather than resting on it alone.</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>FLAGGED: 6-8 weeks is approved only if the body carries the permit dependency.</t>
+          <t>Uses your 6 to 8 week timeline, and carries your own caveat that permit turnaround varies by jurisdiction.</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>PRE-REMODEL ANGLE ONLY. Feeds the finishing service. Never positions ABD as a waterproofing company.</t>
+          <t>A pre-remodel piece that feeds the finishing work. Never positions you as a waterproofing company.</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Use ABD's own project photography. The site explicitly positions its photos against stock imagery.</t>
+          <t>Uses your own project photography. Your site makes a point of this against competitors who buy stock images, so this article should not undercut it.</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>Egress requirement is a code matter. Ties to their existing permits article.</t>
+          <t>Egress is a code requirement, so this links to your existing permits article rather than restating it.</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>Treated bottom plates and moisture-resistant drywall are ABD's published Atlanta baseline.</t>
+          <t>Treated bottom plates and moisture-resistant drywall are already your published baseline for Atlanta's climate. This article follows it.</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="K114" s="6" t="inlineStr">
         <is>
-          <t>PRE-REMODEL ANGLE ONLY.</t>
+          <t>A pre-remodel piece, not a waterproofing service page.</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
       </c>
       <c r="K115" s="6" t="inlineStr">
         <is>
-          <t>PRE-REMODEL ANGLE ONLY. Do not drift into waterproofing services - see brand-facts.md do-NOT-claim.</t>
+          <t>A pre-remodel piece. Stops short of waterproofing services, which you do not sell.</t>
         </is>
       </c>
     </row>
@@ -6092,7 +6092,7 @@
       </c>
       <c r="K116" s="6" t="inlineStr">
         <is>
-          <t>PRE-REMODEL ANGLE ONLY. Highest-volume item in the capped moisture set - keep it educational.</t>
+          <t>The largest item in the small moisture set we kept. Educational throughout, never a pitch for drainage work.</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="K118" s="6" t="inlineStr">
         <is>
-          <t>Their existing permits article pulls national non-buying traffic and 22 municipal .gov competitors. This one must be Georgia-specific to avoid repeating that.</t>
+          <t>Your existing permits article ranks against county government sites nationally and brings in readers who will never hire you. This one stays specific to Georgia so it does not repeat that.</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6240,7 @@
       </c>
       <c r="K119" s="6" t="inlineStr">
         <is>
-          <t>Honest DIY assessment. Do not strawman DIY - the credibility of the whole cluster rests on this one being fair.</t>
+          <t>A genuinely fair assessment of doing it yourself. If this one reads as a sales pitch, it costs the credibility of everything around it.</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6337,7 @@
       </c>
       <c r="K121" s="6" t="inlineStr">
         <is>
-          <t>FLAGGED: permit dependency must appear.</t>
+          <t>Carries your caveat that permit turnaround varies by jurisdiction.</t>
         </is>
       </c>
     </row>
@@ -80298,7 +80298,7 @@
         <is>
           <t>Headlines shown are working titles - the keyword, angle, and funnel stage for each article are locked. Final headlines are SEO-optimized at production, and your input is welcome.
 Month 1 headlines are near-final; they are written before new data can shift them. Months 2 and 3 are our best current targets based on today's data.
-Each month we re-run the plan against live Search Console data. Some articles merge, some get reprioritised, a few get replaced with better opportunities from the Bench tab. That is the plan working, not the plan failing. Every swap comes with a one-line reason in the monthly recap.</t>
+Each month we re-run the plan against live Search Console data. Some articles merge, some get reprioritized, a few get replaced with better opportunities from the Bench tab. That is the plan working, not the plan failing. Every swap comes with a one-line reason in the monthly recap.</t>
         </is>
       </c>
     </row>
@@ -80313,7 +80313,7 @@
       <c r="A30" s="21" t="inlineStr">
         <is>
           <t>Before writing anything, we built a verified facts file from your own live pages: the 5-year warranty and its real scope, your published $45 to $150 per square foot range, the 6 to 8 week timeline, the 3D CAD design process, 26 years in business, and the 30-mile service radius from your Marietta office.
-The 'Writer guardrail' column flags every article where a claim needs care. Your 5-year warranty covers labour, starts at project commencement rather than completion, is non-transferable, and mechanical components carry their own manufacturer warranties. Any article mentioning it has to carry that scope. The 6 to 8 week timeline has to carry the permit dependency. 'Routinely the lowest bid' is your wording and never becomes 'guaranteed lowest'.
+The 'Writer guardrail' column carries a note on 31 of the 120 articles. Most flag a claim that needs care; the rest record a decision worth seeing, such as which city pages have no measured search volume, or which two are on hold pending your answer on service radius. Your 5-year warranty covers labor, starts at project commencement rather than completion, is non-transferable, and mechanical components carry their own manufacturer warranties. Any article mentioning it has to carry that scope. The 6 to 8 week timeline has to carry the permit dependency. 'Routinely the lowest bid' is your wording and never becomes 'guaranteed lowest'.
 Anything we could not verify on your live site is on a do-not-claim list and will not appear in an article. That includes project counts, awards, review ratings, licence numbers and financing terms.</t>
         </is>
       </c>

</xml_diff>